<commit_message>
Generate Taxi Driver packages from app/data and app/templates
Triggered by: fab955b2adc8bcf6556860404367e6cdeb873026
</commit_message>
<xml_diff>
--- a/examples/ltd-latest/Vatreturns.xlsx
+++ b/examples/ltd-latest/Vatreturns.xlsx
@@ -1217,6 +1217,11 @@
       <sheetData sheetId="9"/>
       <sheetData sheetId="10"/>
       <sheetData sheetId="11">
+        <row r="10">
+          <cell r="B10">
+            <v>45777</v>
+          </cell>
+        </row>
         <row r="12">
           <cell r="B12">
             <v>45808</v>
@@ -1350,21 +1355,7 @@
           </cell>
         </row>
       </sheetData>
-      <sheetData sheetId="3">
-        <row r="1">
-          <cell r="G1">
-            <v>0</v>
-          </cell>
-          <cell r="H1">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="4">
-          <cell r="G4">
-            <v>0</v>
-          </cell>
-        </row>
-      </sheetData>
+      <sheetData sheetId="3"/>
       <sheetData sheetId="4"/>
       <sheetData sheetId="5"/>
       <sheetData sheetId="6"/>
@@ -1438,16 +1429,7 @@
           </cell>
         </row>
       </sheetData>
-      <sheetData sheetId="3">
-        <row r="1">
-          <cell r="G1">
-            <v>0</v>
-          </cell>
-          <cell r="H1">
-            <v>0</v>
-          </cell>
-        </row>
-      </sheetData>
+      <sheetData sheetId="3"/>
       <sheetData sheetId="4"/>
       <sheetData sheetId="5"/>
       <sheetData sheetId="6"/>
@@ -1622,7 +1604,7 @@
       <c r="I2" s="14"/>
       <c r="K2" s="15" t="n">
         <f aca="false">Vatinterface!B6</f>
-        <v>45869</v>
+        <v>45838</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1639,7 +1621,7 @@
       <c r="I3" s="14"/>
       <c r="K3" s="15" t="n">
         <f aca="false">Vatinterface!B7</f>
-        <v>45900</v>
+        <v>45869</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1656,7 +1638,7 @@
       <c r="I4" s="14"/>
       <c r="K4" s="15" t="n">
         <f aca="false">Vatinterface!B8</f>
-        <v>45930</v>
+        <v>45900</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1669,13 +1651,13 @@
       </c>
       <c r="F5" s="26"/>
       <c r="G5" s="27" t="n">
-        <v>46295</v>
+        <v>46265</v>
       </c>
       <c r="H5" s="13"/>
       <c r="I5" s="14"/>
       <c r="K5" s="15" t="n">
         <f aca="false">Vatinterface!B9</f>
-        <v>45961</v>
+        <v>45930</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1690,7 +1672,7 @@
       <c r="I6" s="14"/>
       <c r="K6" s="15" t="n">
         <f aca="false">Vatinterface!B10</f>
-        <v>45991</v>
+        <v>45961</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1710,7 +1692,7 @@
       <c r="I7" s="14"/>
       <c r="K7" s="15" t="n">
         <f aca="false">Vatinterface!B11</f>
-        <v>46022</v>
+        <v>45991</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1725,7 +1707,7 @@
       <c r="I8" s="14"/>
       <c r="K8" s="15" t="n">
         <f aca="false">Vatinterface!B12</f>
-        <v>46053</v>
+        <v>46022</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1747,7 +1729,7 @@
       <c r="I9" s="14"/>
       <c r="K9" s="15" t="n">
         <f aca="false">Vatinterface!B13</f>
-        <v>46081</v>
+        <v>46053</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1762,7 +1744,7 @@
       <c r="I10" s="14"/>
       <c r="K10" s="15" t="n">
         <f aca="false">Vatinterface!B14</f>
-        <v>46112</v>
+        <v>46081</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1783,7 +1765,7 @@
       <c r="I11" s="14"/>
       <c r="K11" s="15" t="n">
         <f aca="false">Vatinterface!B15</f>
-        <v>46142</v>
+        <v>46112</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1798,7 +1780,7 @@
       <c r="I12" s="14"/>
       <c r="K12" s="15" t="n">
         <f aca="false">Vatinterface!B16</f>
-        <v>46173</v>
+        <v>46142</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1820,7 +1802,7 @@
       <c r="I13" s="14"/>
       <c r="K13" s="15" t="n">
         <f aca="false">Vatinterface!B17</f>
-        <v>46203</v>
+        <v>46173</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1835,7 +1817,7 @@
       <c r="I14" s="14"/>
       <c r="K14" s="15" t="n">
         <f aca="false">Vatinterface!B18</f>
-        <v>0</v>
+        <v>46203</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -13426,7 +13408,7 @@
       <c r="I2" s="14"/>
       <c r="K2" s="15" t="n">
         <f aca="false">Vatinterface!B6</f>
-        <v>45869</v>
+        <v>45838</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13443,7 +13425,7 @@
       <c r="I3" s="14"/>
       <c r="K3" s="15" t="n">
         <f aca="false">Vatinterface!B7</f>
-        <v>45900</v>
+        <v>45869</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -13460,7 +13442,7 @@
       <c r="I4" s="14"/>
       <c r="K4" s="15" t="n">
         <f aca="false">Vatinterface!B8</f>
-        <v>45930</v>
+        <v>45900</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13473,13 +13455,13 @@
       </c>
       <c r="F5" s="26"/>
       <c r="G5" s="27" t="n">
-        <v>46387</v>
+        <v>46356</v>
       </c>
       <c r="H5" s="13"/>
       <c r="I5" s="14"/>
       <c r="K5" s="15" t="n">
         <f aca="false">Vatinterface!B9</f>
-        <v>45961</v>
+        <v>45930</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -13494,7 +13476,7 @@
       <c r="I6" s="14"/>
       <c r="K6" s="15" t="n">
         <f aca="false">Vatinterface!B10</f>
-        <v>45991</v>
+        <v>45961</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -13514,7 +13496,7 @@
       <c r="I7" s="14"/>
       <c r="K7" s="15" t="n">
         <f aca="false">Vatinterface!B11</f>
-        <v>46022</v>
+        <v>45991</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13529,7 +13511,7 @@
       <c r="I8" s="14"/>
       <c r="K8" s="15" t="n">
         <f aca="false">Vatinterface!B12</f>
-        <v>46053</v>
+        <v>46022</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -13551,7 +13533,7 @@
       <c r="I9" s="14"/>
       <c r="K9" s="15" t="n">
         <f aca="false">Vatinterface!B13</f>
-        <v>46081</v>
+        <v>46053</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -13566,7 +13548,7 @@
       <c r="I10" s="14"/>
       <c r="K10" s="15" t="n">
         <f aca="false">Vatinterface!B14</f>
-        <v>46112</v>
+        <v>46081</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -13587,7 +13569,7 @@
       <c r="I11" s="14"/>
       <c r="K11" s="15" t="n">
         <f aca="false">Vatinterface!B15</f>
-        <v>46142</v>
+        <v>46112</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -13602,7 +13584,7 @@
       <c r="I12" s="14"/>
       <c r="K12" s="15" t="n">
         <f aca="false">Vatinterface!B16</f>
-        <v>46173</v>
+        <v>46142</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -13624,7 +13606,7 @@
       <c r="I13" s="14"/>
       <c r="K13" s="15" t="n">
         <f aca="false">Vatinterface!B17</f>
-        <v>46203</v>
+        <v>46173</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -13639,7 +13621,7 @@
       <c r="I14" s="14"/>
       <c r="K14" s="15" t="n">
         <f aca="false">Vatinterface!B18</f>
-        <v>0</v>
+        <v>46203</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -13990,7 +13972,7 @@
       <c r="I2" s="14"/>
       <c r="K2" s="15" t="n">
         <f aca="false">Vatinterface!B6</f>
-        <v>45869</v>
+        <v>45838</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14007,7 +13989,7 @@
       <c r="I3" s="14"/>
       <c r="K3" s="15" t="n">
         <f aca="false">Vatinterface!B7</f>
-        <v>45900</v>
+        <v>45869</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -14024,7 +14006,7 @@
       <c r="I4" s="14"/>
       <c r="K4" s="15" t="n">
         <f aca="false">Vatinterface!B8</f>
-        <v>45930</v>
+        <v>45900</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14037,13 +14019,13 @@
       </c>
       <c r="F5" s="26"/>
       <c r="G5" s="27" t="n">
-        <v>46477</v>
+        <v>46446</v>
       </c>
       <c r="H5" s="13"/>
       <c r="I5" s="14"/>
       <c r="K5" s="15" t="n">
         <f aca="false">Vatinterface!B9</f>
-        <v>45961</v>
+        <v>45930</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -14058,7 +14040,7 @@
       <c r="I6" s="14"/>
       <c r="K6" s="15" t="n">
         <f aca="false">Vatinterface!B10</f>
-        <v>45991</v>
+        <v>45961</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -14078,7 +14060,7 @@
       <c r="I7" s="14"/>
       <c r="K7" s="15" t="n">
         <f aca="false">Vatinterface!B11</f>
-        <v>46022</v>
+        <v>45991</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14093,7 +14075,7 @@
       <c r="I8" s="14"/>
       <c r="K8" s="15" t="n">
         <f aca="false">Vatinterface!B12</f>
-        <v>46053</v>
+        <v>46022</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -14115,7 +14097,7 @@
       <c r="I9" s="14"/>
       <c r="K9" s="15" t="n">
         <f aca="false">Vatinterface!B13</f>
-        <v>46081</v>
+        <v>46053</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -14130,7 +14112,7 @@
       <c r="I10" s="14"/>
       <c r="K10" s="15" t="n">
         <f aca="false">Vatinterface!B14</f>
-        <v>46112</v>
+        <v>46081</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -14151,7 +14133,7 @@
       <c r="I11" s="14"/>
       <c r="K11" s="15" t="n">
         <f aca="false">Vatinterface!B15</f>
-        <v>46142</v>
+        <v>46112</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -14166,7 +14148,7 @@
       <c r="I12" s="14"/>
       <c r="K12" s="15" t="n">
         <f aca="false">Vatinterface!B16</f>
-        <v>46173</v>
+        <v>46142</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -14188,7 +14170,7 @@
       <c r="I13" s="14"/>
       <c r="K13" s="15" t="n">
         <f aca="false">Vatinterface!B17</f>
-        <v>46203</v>
+        <v>46173</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -14203,7 +14185,7 @@
       <c r="I14" s="14"/>
       <c r="K14" s="15" t="n">
         <f aca="false">Vatinterface!B18</f>
-        <v>0</v>
+        <v>46203</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -14554,7 +14536,7 @@
       <c r="I2" s="14"/>
       <c r="K2" s="15" t="n">
         <f aca="false">Vatinterface!B6</f>
-        <v>45869</v>
+        <v>45838</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14571,7 +14553,7 @@
       <c r="I3" s="14"/>
       <c r="K3" s="15" t="n">
         <f aca="false">Vatinterface!B7</f>
-        <v>45900</v>
+        <v>45869</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -14588,7 +14570,7 @@
       <c r="I4" s="14"/>
       <c r="K4" s="15" t="n">
         <f aca="false">Vatinterface!B8</f>
-        <v>45930</v>
+        <v>45900</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14601,13 +14583,13 @@
       </c>
       <c r="F5" s="26"/>
       <c r="G5" s="27" t="n">
-        <v>46568</v>
+        <v>46538</v>
       </c>
       <c r="H5" s="13"/>
       <c r="I5" s="14"/>
       <c r="K5" s="15" t="n">
         <f aca="false">Vatinterface!B9</f>
-        <v>45961</v>
+        <v>45930</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -14622,7 +14604,7 @@
       <c r="I6" s="14"/>
       <c r="K6" s="15" t="n">
         <f aca="false">Vatinterface!B10</f>
-        <v>45991</v>
+        <v>45961</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -14642,7 +14624,7 @@
       <c r="I7" s="14"/>
       <c r="K7" s="15" t="n">
         <f aca="false">Vatinterface!B11</f>
-        <v>46022</v>
+        <v>45991</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14657,7 +14639,7 @@
       <c r="I8" s="14"/>
       <c r="K8" s="15" t="n">
         <f aca="false">Vatinterface!B12</f>
-        <v>46053</v>
+        <v>46022</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -14679,7 +14661,7 @@
       <c r="I9" s="14"/>
       <c r="K9" s="15" t="n">
         <f aca="false">Vatinterface!B13</f>
-        <v>46081</v>
+        <v>46053</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -14694,7 +14676,7 @@
       <c r="I10" s="14"/>
       <c r="K10" s="15" t="n">
         <f aca="false">Vatinterface!B14</f>
-        <v>46112</v>
+        <v>46081</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -14715,7 +14697,7 @@
       <c r="I11" s="14"/>
       <c r="K11" s="15" t="n">
         <f aca="false">Vatinterface!B15</f>
-        <v>46142</v>
+        <v>46112</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -14730,7 +14712,7 @@
       <c r="I12" s="14"/>
       <c r="K12" s="15" t="n">
         <f aca="false">Vatinterface!B16</f>
-        <v>46173</v>
+        <v>46142</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -14752,7 +14734,7 @@
       <c r="I13" s="14"/>
       <c r="K13" s="15" t="n">
         <f aca="false">Vatinterface!B17</f>
-        <v>46203</v>
+        <v>46173</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -14767,7 +14749,7 @@
       <c r="I14" s="14"/>
       <c r="K14" s="15" t="n">
         <f aca="false">Vatinterface!B18</f>
-        <v>0</v>
+        <v>46203</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -15118,7 +15100,7 @@
       <c r="I2" s="14"/>
       <c r="K2" s="15" t="n">
         <f aca="false">Vatinterface!B6</f>
-        <v>45869</v>
+        <v>45838</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15135,7 +15117,7 @@
       <c r="I3" s="14"/>
       <c r="K3" s="15" t="n">
         <f aca="false">Vatinterface!B7</f>
-        <v>45900</v>
+        <v>45869</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -15152,7 +15134,7 @@
       <c r="I4" s="14"/>
       <c r="K4" s="15" t="n">
         <f aca="false">Vatinterface!B8</f>
-        <v>45930</v>
+        <v>45900</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15165,13 +15147,13 @@
       </c>
       <c r="F5" s="26"/>
       <c r="G5" s="27" t="n">
-        <v>46599</v>
+        <v>46568</v>
       </c>
       <c r="H5" s="13"/>
       <c r="I5" s="14"/>
       <c r="K5" s="15" t="n">
         <f aca="false">Vatinterface!B9</f>
-        <v>45961</v>
+        <v>45930</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -15186,7 +15168,7 @@
       <c r="I6" s="14"/>
       <c r="K6" s="15" t="n">
         <f aca="false">Vatinterface!B10</f>
-        <v>45991</v>
+        <v>45961</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -15206,7 +15188,7 @@
       <c r="I7" s="14"/>
       <c r="K7" s="15" t="n">
         <f aca="false">Vatinterface!B11</f>
-        <v>46022</v>
+        <v>45991</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15221,7 +15203,7 @@
       <c r="I8" s="14"/>
       <c r="K8" s="15" t="n">
         <f aca="false">Vatinterface!B12</f>
-        <v>46053</v>
+        <v>46022</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -15243,7 +15225,7 @@
       <c r="I9" s="14"/>
       <c r="K9" s="15" t="n">
         <f aca="false">Vatinterface!B13</f>
-        <v>46081</v>
+        <v>46053</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -15258,7 +15240,7 @@
       <c r="I10" s="14"/>
       <c r="K10" s="15" t="n">
         <f aca="false">Vatinterface!B14</f>
-        <v>46112</v>
+        <v>46081</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -15279,7 +15261,7 @@
       <c r="I11" s="14"/>
       <c r="K11" s="15" t="n">
         <f aca="false">Vatinterface!B15</f>
-        <v>46142</v>
+        <v>46112</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -15294,7 +15276,7 @@
       <c r="I12" s="14"/>
       <c r="K12" s="15" t="n">
         <f aca="false">Vatinterface!B16</f>
-        <v>46173</v>
+        <v>46142</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -15316,7 +15298,7 @@
       <c r="I13" s="14"/>
       <c r="K13" s="15" t="n">
         <f aca="false">Vatinterface!B17</f>
-        <v>46203</v>
+        <v>46173</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -15331,7 +15313,7 @@
       <c r="I14" s="14"/>
       <c r="K14" s="15" t="n">
         <f aca="false">Vatinterface!B18</f>
-        <v>0</v>
+        <v>46203</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -15725,12 +15707,12 @@
     <row r="4" customFormat="false" ht="12" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="84"/>
       <c r="B4" s="85" t="n">
-        <f aca="false">[1]Admin!$B$12</f>
-        <v>45808</v>
+        <f aca="false">[1]Admin!$B$10</f>
+        <v>45777</v>
       </c>
       <c r="C4" s="85" t="n">
         <f aca="false">B5</f>
-        <v>45838</v>
+        <v>45808</v>
       </c>
       <c r="D4" s="86" t="n">
         <f aca="false">S02Y1!$H$1</f>
@@ -15762,12 +15744,12 @@
     <row r="5" customFormat="false" ht="12" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="84"/>
       <c r="B5" s="85" t="n">
-        <f aca="false">[1]Admin!$B$14</f>
-        <v>45838</v>
+        <f aca="false">[1]Admin!$B$12</f>
+        <v>45808</v>
       </c>
       <c r="C5" s="85" t="n">
         <f aca="false">B6</f>
-        <v>45869</v>
+        <v>45838</v>
       </c>
       <c r="D5" s="86" t="n">
         <f aca="false">S03Y1!$H$1</f>
@@ -15799,12 +15781,12 @@
     <row r="6" customFormat="false" ht="12" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="84"/>
       <c r="B6" s="85" t="n">
-        <f aca="false">[1]Admin!$B$16</f>
-        <v>45869</v>
+        <f aca="false">[1]Admin!$B$14</f>
+        <v>45838</v>
       </c>
       <c r="C6" s="85" t="n">
         <f aca="false">B7</f>
-        <v>45900</v>
+        <v>45869</v>
       </c>
       <c r="D6" s="86" t="n">
         <f aca="false">[2]Apr!$H$1</f>
@@ -15848,12 +15830,12 @@
     <row r="7" customFormat="false" ht="12" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="84"/>
       <c r="B7" s="85" t="n">
-        <f aca="false">[1]Admin!$B$18</f>
-        <v>45900</v>
+        <f aca="false">[1]Admin!$B$16</f>
+        <v>45869</v>
       </c>
       <c r="C7" s="85" t="n">
         <f aca="false">B8</f>
-        <v>45930</v>
+        <v>45900</v>
       </c>
       <c r="D7" s="86" t="n">
         <f aca="false">[2]May!$H$1</f>
@@ -15897,15 +15879,15 @@
     <row r="8" customFormat="false" ht="12" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="84"/>
       <c r="B8" s="85" t="n">
-        <f aca="false">[1]Admin!$B$20</f>
-        <v>45930</v>
+        <f aca="false">[1]Admin!$B$18</f>
+        <v>45900</v>
       </c>
       <c r="C8" s="85" t="n">
         <f aca="false">B9</f>
-        <v>45961</v>
+        <v>45930</v>
       </c>
       <c r="D8" s="86" t="n">
-        <f aca="false">[2]Jun!$H$1</f>
+        <f aca="false">[2]Apr!$H$1</f>
         <v>0</v>
       </c>
       <c r="E8" s="87" t="n">
@@ -15913,7 +15895,7 @@
         <v>0</v>
       </c>
       <c r="F8" s="87" t="n">
-        <f aca="false">[2]Jun!$G$1</f>
+        <f aca="false">[2]Apr!$G$1</f>
         <v>0</v>
       </c>
       <c r="G8" s="87" t="n">
@@ -15921,7 +15903,7 @@
         <v>0</v>
       </c>
       <c r="H8" s="87" t="n">
-        <f aca="false">[3]Jun!$H$1</f>
+        <f aca="false">[3]Apr!$H$1</f>
         <v>0</v>
       </c>
       <c r="I8" s="87" t="n">
@@ -15929,7 +15911,7 @@
         <v>0</v>
       </c>
       <c r="J8" s="87" t="n">
-        <f aca="false">[3]Jun!$G$1</f>
+        <f aca="false">[3]Apr!$G$1</f>
         <v>0</v>
       </c>
       <c r="K8" s="87" t="n">
@@ -15938,7 +15920,7 @@
       </c>
       <c r="L8" s="88"/>
       <c r="M8" s="89" t="n">
-        <f aca="false">IF([2]Jun!$G$4&gt;0,[2]Jun!$G$4,0)</f>
+        <f aca="false">IF([2]May!$G$4&gt;0,[2]May!$G$4,0)</f>
         <v>0</v>
       </c>
       <c r="N8" s="90"/>
@@ -15946,15 +15928,15 @@
     <row r="9" customFormat="false" ht="12" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="84"/>
       <c r="B9" s="85" t="n">
-        <f aca="false">[1]Admin!$B$22</f>
-        <v>45961</v>
+        <f aca="false">[1]Admin!$B$20</f>
+        <v>45930</v>
       </c>
       <c r="C9" s="85" t="n">
         <f aca="false">B10</f>
-        <v>45991</v>
+        <v>45961</v>
       </c>
       <c r="D9" s="86" t="n">
-        <f aca="false">[2]Apr!$H$1</f>
+        <f aca="false">[2]May!$H$1</f>
         <v>0</v>
       </c>
       <c r="E9" s="87" t="n">
@@ -15962,7 +15944,7 @@
         <v>0</v>
       </c>
       <c r="F9" s="87" t="n">
-        <f aca="false">[2]Apr!$G$1</f>
+        <f aca="false">[2]May!$G$1</f>
         <v>0</v>
       </c>
       <c r="G9" s="87" t="n">
@@ -15970,7 +15952,7 @@
         <v>0</v>
       </c>
       <c r="H9" s="87" t="n">
-        <f aca="false">[3]Apr!$H$1</f>
+        <f aca="false">[3]May!$H$1</f>
         <v>0</v>
       </c>
       <c r="I9" s="87" t="n">
@@ -15978,7 +15960,7 @@
         <v>0</v>
       </c>
       <c r="J9" s="87" t="n">
-        <f aca="false">[3]Apr!$G$1</f>
+        <f aca="false">[3]May!$G$1</f>
         <v>0</v>
       </c>
       <c r="K9" s="87" t="n">
@@ -15995,15 +15977,15 @@
     <row r="10" customFormat="false" ht="12" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="84"/>
       <c r="B10" s="85" t="n">
-        <f aca="false">[1]Admin!$B$24</f>
-        <v>45991</v>
+        <f aca="false">[1]Admin!$B$22</f>
+        <v>45961</v>
       </c>
       <c r="C10" s="85" t="n">
         <f aca="false">B11</f>
-        <v>46022</v>
+        <v>45991</v>
       </c>
       <c r="D10" s="86" t="n">
-        <f aca="false">[2]May!$H$1</f>
+        <f aca="false">[2]Apr!$H$1</f>
         <v>0</v>
       </c>
       <c r="E10" s="87" t="n">
@@ -16011,7 +15993,7 @@
         <v>0</v>
       </c>
       <c r="F10" s="87" t="n">
-        <f aca="false">[2]May!$G$1</f>
+        <f aca="false">[2]Apr!$G$1</f>
         <v>0</v>
       </c>
       <c r="G10" s="87" t="n">
@@ -16019,7 +16001,7 @@
         <v>0</v>
       </c>
       <c r="H10" s="87" t="n">
-        <f aca="false">[3]May!$H$1</f>
+        <f aca="false">[3]Apr!$H$1</f>
         <v>0</v>
       </c>
       <c r="I10" s="87" t="n">
@@ -16027,7 +16009,7 @@
         <v>0</v>
       </c>
       <c r="J10" s="87" t="n">
-        <f aca="false">[3]May!$G$1</f>
+        <f aca="false">[3]Apr!$G$1</f>
         <v>0</v>
       </c>
       <c r="K10" s="87" t="n">
@@ -16036,7 +16018,7 @@
       </c>
       <c r="L10" s="88"/>
       <c r="M10" s="89" t="n">
-        <f aca="false">IF([2]Jun!$G$4&gt;0,[2]Jun!$G$4,0)</f>
+        <f aca="false">IF([2]May!$G$4&gt;0,[2]May!$G$4,0)</f>
         <v>0</v>
       </c>
       <c r="N10" s="90"/>
@@ -16044,15 +16026,15 @@
     <row r="11" customFormat="false" ht="12" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="84"/>
       <c r="B11" s="85" t="n">
-        <f aca="false">[1]Admin!$B$26</f>
-        <v>46022</v>
+        <f aca="false">[1]Admin!$B$24</f>
+        <v>45991</v>
       </c>
       <c r="C11" s="85" t="n">
         <f aca="false">B12</f>
-        <v>46053</v>
+        <v>46022</v>
       </c>
       <c r="D11" s="86" t="n">
-        <f aca="false">[2]Jun!$H$1</f>
+        <f aca="false">[2]May!$H$1</f>
         <v>0</v>
       </c>
       <c r="E11" s="87" t="n">
@@ -16060,7 +16042,7 @@
         <v>0</v>
       </c>
       <c r="F11" s="87" t="n">
-        <f aca="false">[2]Jun!$G$1</f>
+        <f aca="false">[2]May!$G$1</f>
         <v>0</v>
       </c>
       <c r="G11" s="87" t="n">
@@ -16068,7 +16050,7 @@
         <v>0</v>
       </c>
       <c r="H11" s="87" t="n">
-        <f aca="false">[3]Jun!$H$1</f>
+        <f aca="false">[3]May!$H$1</f>
         <v>0</v>
       </c>
       <c r="I11" s="87" t="n">
@@ -16076,7 +16058,7 @@
         <v>0</v>
       </c>
       <c r="J11" s="87" t="n">
-        <f aca="false">[3]Jun!$G$1</f>
+        <f aca="false">[3]May!$G$1</f>
         <v>0</v>
       </c>
       <c r="K11" s="87" t="n">
@@ -16085,7 +16067,7 @@
       </c>
       <c r="L11" s="88"/>
       <c r="M11" s="89" t="n">
-        <f aca="false">IF([2]Jun!$G$4&gt;0,[2]Jun!$G$4,0)</f>
+        <f aca="false">IF([2]Apr!$G$4&gt;0,[2]Apr!$G$4,0)</f>
         <v>0</v>
       </c>
       <c r="N11" s="90"/>
@@ -16093,12 +16075,12 @@
     <row r="12" customFormat="false" ht="12" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="84"/>
       <c r="B12" s="85" t="n">
-        <f aca="false">[1]Admin!$B$28</f>
-        <v>46053</v>
+        <f aca="false">[1]Admin!$B$26</f>
+        <v>46022</v>
       </c>
       <c r="C12" s="85" t="n">
         <f aca="false">B13</f>
-        <v>46081</v>
+        <v>46053</v>
       </c>
       <c r="D12" s="86" t="n">
         <f aca="false">[2]Apr!$H$1</f>
@@ -16142,12 +16124,12 @@
     <row r="13" customFormat="false" ht="12" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="84"/>
       <c r="B13" s="85" t="n">
-        <f aca="false">[1]Admin!$B$30</f>
-        <v>46081</v>
+        <f aca="false">[1]Admin!$B$28</f>
+        <v>46053</v>
       </c>
       <c r="C13" s="85" t="n">
         <f aca="false">B14</f>
-        <v>46112</v>
+        <v>46081</v>
       </c>
       <c r="D13" s="86" t="n">
         <f aca="false">[2]May!$H$1</f>
@@ -16183,7 +16165,7 @@
       </c>
       <c r="L13" s="88"/>
       <c r="M13" s="89" t="n">
-        <f aca="false">IF([2]May!$G$4&gt;0,[2]May!$G$4,0)</f>
+        <f aca="false">IF([2]Apr!$G$4&gt;0,[2]Apr!$G$4,0)</f>
         <v>0</v>
       </c>
       <c r="N13" s="90"/>
@@ -16191,15 +16173,15 @@
     <row r="14" customFormat="false" ht="12" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="84"/>
       <c r="B14" s="85" t="n">
-        <f aca="false">[1]Admin!$B$32</f>
-        <v>46112</v>
+        <f aca="false">[1]Admin!$B$30</f>
+        <v>46081</v>
       </c>
       <c r="C14" s="85" t="n">
         <f aca="false">B15</f>
-        <v>46142</v>
+        <v>46112</v>
       </c>
       <c r="D14" s="86" t="n">
-        <f aca="false">[2]Jun!$H$1</f>
+        <f aca="false">[2]Apr!$H$1</f>
         <v>0</v>
       </c>
       <c r="E14" s="87" t="n">
@@ -16207,7 +16189,7 @@
         <v>0</v>
       </c>
       <c r="F14" s="87" t="n">
-        <f aca="false">[2]Jun!$G$1</f>
+        <f aca="false">[2]Apr!$G$1</f>
         <v>0</v>
       </c>
       <c r="G14" s="87" t="n">
@@ -16215,7 +16197,7 @@
         <v>0</v>
       </c>
       <c r="H14" s="87" t="n">
-        <f aca="false">[3]Jun!$H$1</f>
+        <f aca="false">[3]Apr!$H$1</f>
         <v>0</v>
       </c>
       <c r="I14" s="87" t="n">
@@ -16223,7 +16205,7 @@
         <v>0</v>
       </c>
       <c r="J14" s="87" t="n">
-        <f aca="false">[3]Jun!$G$1</f>
+        <f aca="false">[3]Apr!$G$1</f>
         <v>0</v>
       </c>
       <c r="K14" s="87" t="n">
@@ -16232,7 +16214,7 @@
       </c>
       <c r="L14" s="88"/>
       <c r="M14" s="89" t="n">
-        <f aca="false">IF([2]May!$G$4&gt;0,[2]May!$G$4,0)</f>
+        <f aca="false">IF([2]Apr!$G$4&gt;0,[2]Apr!$G$4,0)</f>
         <v>0</v>
       </c>
       <c r="N14" s="90"/>
@@ -16240,15 +16222,15 @@
     <row r="15" customFormat="false" ht="12" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="84"/>
       <c r="B15" s="85" t="n">
-        <f aca="false">[1]Admin!$B$34</f>
-        <v>46142</v>
+        <f aca="false">[1]Admin!$B$32</f>
+        <v>46112</v>
       </c>
       <c r="C15" s="85" t="n">
         <f aca="false">B16</f>
-        <v>46173</v>
+        <v>46142</v>
       </c>
       <c r="D15" s="86" t="n">
-        <f aca="false">[2]Apr!$H$1</f>
+        <f aca="false">[2]May!$H$1</f>
         <v>0</v>
       </c>
       <c r="E15" s="87" t="n">
@@ -16256,7 +16238,7 @@
         <v>0</v>
       </c>
       <c r="F15" s="87" t="n">
-        <f aca="false">[2]Apr!$G$1</f>
+        <f aca="false">[2]May!$G$1</f>
         <v>0</v>
       </c>
       <c r="G15" s="87" t="n">
@@ -16264,7 +16246,7 @@
         <v>0</v>
       </c>
       <c r="H15" s="87" t="n">
-        <f aca="false">[3]Apr!$H$1</f>
+        <f aca="false">[3]May!$H$1</f>
         <v>0</v>
       </c>
       <c r="I15" s="87" t="n">
@@ -16272,7 +16254,7 @@
         <v>0</v>
       </c>
       <c r="J15" s="87" t="n">
-        <f aca="false">[3]Apr!$G$1</f>
+        <f aca="false">[3]May!$G$1</f>
         <v>0</v>
       </c>
       <c r="K15" s="87" t="n">
@@ -16289,15 +16271,15 @@
     <row r="16" customFormat="false" ht="12" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="84"/>
       <c r="B16" s="85" t="n">
-        <f aca="false">[1]Admin!$B$36</f>
-        <v>46173</v>
+        <f aca="false">[1]Admin!$B$34</f>
+        <v>46142</v>
       </c>
       <c r="C16" s="85" t="n">
         <f aca="false">B17</f>
-        <v>46203</v>
+        <v>46173</v>
       </c>
       <c r="D16" s="86" t="n">
-        <f aca="false">[2]May!$H$1</f>
+        <f aca="false">[2]Apr!$H$1</f>
         <v>0</v>
       </c>
       <c r="E16" s="87" t="n">
@@ -16305,7 +16287,7 @@
         <v>0</v>
       </c>
       <c r="F16" s="87" t="n">
-        <f aca="false">[2]May!$G$1</f>
+        <f aca="false">[2]Apr!$G$1</f>
         <v>0</v>
       </c>
       <c r="G16" s="87" t="n">
@@ -16313,7 +16295,7 @@
         <v>0</v>
       </c>
       <c r="H16" s="87" t="n">
-        <f aca="false">[3]May!$H$1</f>
+        <f aca="false">[3]Apr!$H$1</f>
         <v>0</v>
       </c>
       <c r="I16" s="87" t="n">
@@ -16321,7 +16303,7 @@
         <v>0</v>
       </c>
       <c r="J16" s="87" t="n">
-        <f aca="false">[3]May!$G$1</f>
+        <f aca="false">[3]Apr!$G$1</f>
         <v>0</v>
       </c>
       <c r="K16" s="87" t="n">
@@ -16330,7 +16312,7 @@
       </c>
       <c r="L16" s="88"/>
       <c r="M16" s="89" t="n">
-        <f aca="false">IF([2]Jun!$G$4&gt;0,[2]Jun!$G$4,0)</f>
+        <f aca="false">IF([2]Apr!$G$4&gt;0,[2]Apr!$G$4,0)</f>
         <v>0</v>
       </c>
       <c r="N16" s="90"/>
@@ -16338,15 +16320,15 @@
     <row r="17" customFormat="false" ht="12" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="84"/>
       <c r="B17" s="85" t="n">
-        <f aca="false">[1]Admin!$B$38</f>
-        <v>46203</v>
+        <f aca="false">[1]Admin!$B$36</f>
+        <v>46173</v>
       </c>
       <c r="C17" s="85" t="n">
         <f aca="false">B18</f>
-        <v>0</v>
+        <v>46203</v>
       </c>
       <c r="D17" s="86" t="n">
-        <f aca="false">[2]Jun!$H$1</f>
+        <f aca="false">[2]May!$H$1</f>
         <v>0</v>
       </c>
       <c r="E17" s="87" t="n">
@@ -16354,7 +16336,7 @@
         <v>0</v>
       </c>
       <c r="F17" s="87" t="n">
-        <f aca="false">[2]Jun!$G$1</f>
+        <f aca="false">[2]May!$G$1</f>
         <v>0</v>
       </c>
       <c r="G17" s="87" t="n">
@@ -16362,7 +16344,7 @@
         <v>0</v>
       </c>
       <c r="H17" s="87" t="n">
-        <f aca="false">[3]Jun!$H$1</f>
+        <f aca="false">[3]May!$H$1</f>
         <v>0</v>
       </c>
       <c r="I17" s="87" t="n">
@@ -16370,7 +16352,7 @@
         <v>0</v>
       </c>
       <c r="J17" s="87" t="n">
-        <f aca="false">[3]Jun!$G$1</f>
+        <f aca="false">[3]May!$G$1</f>
         <v>0</v>
       </c>
       <c r="K17" s="87" t="n">
@@ -16379,7 +16361,7 @@
       </c>
       <c r="L17" s="88"/>
       <c r="M17" s="89" t="n">
-        <f aca="false">IF([2]Jun!$G$4&gt;0,[2]Jun!$G$4,0)</f>
+        <f aca="false">IF([2]May!$G$4&gt;0,[2]May!$G$4,0)</f>
         <v>0</v>
       </c>
       <c r="N17" s="90"/>
@@ -16387,8 +16369,8 @@
     <row r="18" customFormat="false" ht="12" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="84"/>
       <c r="B18" s="85" t="n">
-        <f aca="false">[1]Admin!$B$40</f>
-        <v>0</v>
+        <f aca="false">[1]Admin!$B$38</f>
+        <v>46203</v>
       </c>
       <c r="C18" s="85" t="n">
         <f aca="false">B19</f>
@@ -16428,7 +16410,7 @@
       </c>
       <c r="L18" s="88"/>
       <c r="M18" s="89" t="n">
-        <f aca="false">IF([2]Jun!$G$4&gt;0,[2]Jun!$G$4,0)</f>
+        <f aca="false">IF([2]May!$G$4&gt;0,[2]May!$G$4,0)</f>
         <v>0</v>
       </c>
       <c r="N18" s="90"/>
@@ -16436,7 +16418,7 @@
     <row r="19" customFormat="false" ht="12" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="84"/>
       <c r="B19" s="85" t="n">
-        <f aca="false">[1]Admin!$B$42</f>
+        <f aca="false">[1]Admin!$B$40</f>
         <v>0</v>
       </c>
       <c r="C19" s="91" t="n">
@@ -16477,7 +16459,7 @@
       </c>
       <c r="L19" s="88"/>
       <c r="M19" s="89" t="n">
-        <f aca="false">IF([2]Jun!$G$4&gt;0,[2]Jun!$G$4,0)</f>
+        <f aca="false">IF([2]May!$G$4&gt;0,[2]May!$G$4,0)</f>
         <v>0</v>
       </c>
       <c r="N19" s="90"/>

</xml_diff>